<commit_message>
Checkpoint 2: planted answers and pilot pack rendered and critiqued; critique fixes; renderer, numbers and CSV improvements
</commit_message>
<xml_diff>
--- a/output/archive/BrindlewytheData/Studies/2011/BW11_0275/Results/BW11_0275_hERG-CYP_RUN04.xlsx
+++ b/output/archive/BrindlewytheData/Studies/2011/BW11_0275/Results/BW11_0275_hERG-CYP_RUN04.xlsx
@@ -174,7 +174,7 @@
   <commentList>
     <comment ref="E3" authorId="0" shapeId="0">
       <text>
-        <t>Geometric mean of accepted cells; censored replicates excluded</t>
+        <t>Geometric mean of finite cell IC50s when they are the majority of accepted cells; otherwise &gt;30 µM (&gt;10 µM where precipitation limited the top concentration). n = accepted cells (finite).</t>
       </text>
     </comment>
   </commentList>
@@ -528,13 +528,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -551,6 +551,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -590,12 +591,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Study Director</t>
+          <t>Study lead</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Dr A. Veldershain</t>
+          <t>Dr A. Veldershain (Study Director)</t>
         </is>
       </c>
     </row>
@@ -673,10 +674,11 @@
         <v>0.029</v>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>Study summary (benchmark)</t>
+          <t>Study summary</t>
         </is>
       </c>
     </row>
@@ -898,6 +900,7 @@
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -905,28 +908,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="13.5" customWidth="1" min="2" max="2"/>
-    <col width="13.5" customWidth="1" min="3" max="3"/>
-    <col width="13.5" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="17.1" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="18.8" customWidth="1" min="2" max="2"/>
+    <col width="18.8" customWidth="1" min="3" max="3"/>
+    <col width="18.8" customWidth="1" min="4" max="4"/>
+    <col width="19.85" customWidth="1" min="5" max="5"/>
+    <col width="21.95" customWidth="1" min="6" max="6"/>
+    <col width="18.8" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>hERG automated patch clamp: tail-current IC50, 6-point, top 30 µM</t>
-        </is>
-      </c>
-    </row>
+          <t>hERG automated patch clamp: tail-current IC50 per cell, 6-point, top 30 µM</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -935,22 +939,22 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>IC50 rep 1 (µM)</t>
+          <t>IC50 cell 1 (µM)</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>IC50 rep 2 (µM)</t>
+          <t>IC50 cell 2 (µM)</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>IC50 rep 3 (µM)</t>
+          <t>IC50 cell 3 (µM)</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>IC50 mean (µM)</t>
+          <t>IC50 geomean (µM)</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -960,7 +964,7 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>n cells (finite)</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -990,8 +994,10 @@
       <c r="F4" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="G4" s="2" t="n">
-        <v>3</v>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>3 (3)</t>
+        </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
     </row>
@@ -1016,8 +1022,10 @@
       <c r="F5" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G5" s="2" t="n">
-        <v>3</v>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>3 (3)</t>
+        </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
     </row>
@@ -1040,8 +1048,10 @@
       <c r="F6" s="2" t="n">
         <v>86</v>
       </c>
-      <c r="G6" s="2" t="n">
-        <v>2</v>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
     </row>
@@ -1066,8 +1076,10 @@
       <c r="F7" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="G7" s="2" t="n">
-        <v>3</v>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>3 (3)</t>
+        </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
     </row>
@@ -1090,8 +1102,10 @@
       <c r="F8" s="2" t="n">
         <v>37</v>
       </c>
-      <c r="G8" s="2" t="n">
-        <v>2</v>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
     </row>
@@ -1118,8 +1132,10 @@
       <c r="F9" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="G9" s="2" t="n">
-        <v>2</v>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>2 (1)</t>
+        </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
     </row>
@@ -1142,8 +1158,10 @@
       <c r="F10" s="2" t="n">
         <v>61</v>
       </c>
-      <c r="G10" s="2" t="n">
-        <v>2</v>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
     </row>
@@ -1166,12 +1184,14 @@
       <c r="F11" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="G11" s="2" t="n">
-        <v>2</v>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Run 2 rejected (E-4031 outside range); repeated</t>
+          <t>First run rejected (E-4031 outside range); repeated</t>
         </is>
       </c>
     </row>
@@ -1194,12 +1214,14 @@
       <c r="F12" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="G12" s="2" t="n">
-        <v>2</v>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Run 2 rejected (E-4031 outside range); repeated</t>
+          <t>First run rejected (E-4031 outside range); repeated</t>
         </is>
       </c>
     </row>
@@ -1222,8 +1244,10 @@
       <c r="F13" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="G13" s="2" t="n">
-        <v>2</v>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
     </row>
@@ -1246,8 +1270,10 @@
       <c r="F14" s="2" t="n">
         <v>69</v>
       </c>
-      <c r="G14" s="2" t="n">
-        <v>2</v>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
     </row>
@@ -1270,8 +1296,10 @@
       <c r="F15" s="2" t="n">
         <v>69</v>
       </c>
-      <c r="G15" s="2" t="n">
-        <v>2</v>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H15" s="2" t="inlineStr"/>
     </row>
@@ -1294,8 +1322,10 @@
       <c r="F16" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="G16" s="2" t="n">
-        <v>2</v>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
     </row>
@@ -1320,8 +1350,10 @@
       <c r="F17" s="2" t="n">
         <v>54</v>
       </c>
-      <c r="G17" s="2" t="n">
-        <v>3</v>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>3 (3)</t>
+        </is>
       </c>
       <c r="H17" s="2" t="inlineStr"/>
     </row>
@@ -1344,8 +1376,10 @@
       <c r="F18" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="G18" s="2" t="n">
-        <v>2</v>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
     </row>
@@ -1368,8 +1402,10 @@
       <c r="F19" s="2" t="n">
         <v>66</v>
       </c>
-      <c r="G19" s="2" t="n">
-        <v>2</v>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
     </row>
@@ -1394,8 +1430,10 @@
       <c r="F20" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="G20" s="2" t="n">
-        <v>3</v>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>3 (3)</t>
+        </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
     </row>
@@ -1418,8 +1456,10 @@
       <c r="F21" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="G21" s="2" t="n">
-        <v>2</v>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
     </row>
@@ -1442,8 +1482,10 @@
       <c r="F22" s="2" t="n">
         <v>80</v>
       </c>
-      <c r="G22" s="2" t="n">
-        <v>2</v>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
     </row>
@@ -1466,8 +1508,10 @@
       <c r="F23" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="G23" s="2" t="n">
-        <v>2</v>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
     </row>
@@ -1490,8 +1534,10 @@
       <c r="F24" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="G24" s="2" t="n">
-        <v>2</v>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
     </row>
@@ -1514,8 +1560,10 @@
       <c r="F25" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="G25" s="2" t="n">
-        <v>2</v>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H25" s="2" t="inlineStr"/>
     </row>
@@ -1542,8 +1590,10 @@
       <c r="F26" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="G26" s="2" t="n">
-        <v>2</v>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>2 (1)</t>
+        </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
     </row>
@@ -1566,8 +1616,10 @@
       <c r="F27" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="G27" s="2" t="n">
-        <v>2</v>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
     </row>
@@ -1590,8 +1642,10 @@
       <c r="F28" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="G28" s="2" t="n">
-        <v>2</v>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
     </row>
@@ -1614,8 +1668,10 @@
       <c r="F29" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="G29" s="2" t="n">
-        <v>2</v>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
     </row>
@@ -1642,8 +1698,10 @@
       <c r="F30" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="G30" s="2" t="n">
-        <v>2</v>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>2 (1)</t>
+        </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
     </row>
@@ -1666,8 +1724,10 @@
       <c r="F31" s="2" t="n">
         <v>74</v>
       </c>
-      <c r="G31" s="2" t="n">
-        <v>2</v>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
     </row>
@@ -1692,8 +1752,10 @@
       <c r="F32" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="G32" s="2" t="n">
-        <v>3</v>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>3 (3)</t>
+        </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
     </row>
@@ -1716,8 +1778,10 @@
       <c r="F33" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="G33" s="2" t="n">
-        <v>2</v>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H33" s="2" t="inlineStr"/>
     </row>
@@ -1740,8 +1804,10 @@
       <c r="F34" s="2" t="n">
         <v>57</v>
       </c>
-      <c r="G34" s="2" t="n">
-        <v>2</v>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
     </row>
@@ -1764,8 +1830,10 @@
       <c r="F35" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="G35" s="2" t="n">
-        <v>2</v>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H35" s="2" t="inlineStr"/>
     </row>
@@ -1790,8 +1858,10 @@
       <c r="F36" s="2" t="n">
         <v>78</v>
       </c>
-      <c r="G36" s="2" t="n">
-        <v>3</v>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>3 (3)</t>
+        </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
     </row>
@@ -1814,8 +1884,10 @@
       <c r="F37" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="G37" s="2" t="n">
-        <v>2</v>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H37" s="2" t="inlineStr"/>
     </row>
@@ -1838,8 +1910,10 @@
       <c r="F38" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="G38" s="2" t="n">
-        <v>2</v>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
     </row>
@@ -1862,8 +1936,10 @@
       <c r="F39" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="G39" s="2" t="n">
-        <v>2</v>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
     </row>
@@ -1886,12 +1962,14 @@
       <c r="F40" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="G40" s="2" t="n">
-        <v>2</v>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Run 2 rejected (E-4031 outside range); repeated</t>
+          <t>First run rejected (E-4031 outside range); repeated</t>
         </is>
       </c>
     </row>
@@ -1914,8 +1992,10 @@
       <c r="F41" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="G41" s="2" t="n">
-        <v>2</v>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
     </row>
@@ -1938,8 +2018,10 @@
       <c r="F42" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="G42" s="2" t="n">
-        <v>2</v>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
     </row>
@@ -1962,11 +2044,14 @@
       <c r="F43" s="2" t="n">
         <v>47</v>
       </c>
-      <c r="G43" s="2" t="n">
-        <v>2</v>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>2 (2)</t>
+        </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
     </row>
+    <row r="44"/>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
@@ -1974,8 +2059,16 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Compound IC50 = geometric mean of finite cell IC50s when they are the majority of accepted cells; otherwise reported as &gt;30 µM (or &gt;10 µM where solubility-limited)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -1985,15 +2078,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13.55" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
@@ -2005,6 +2098,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -2917,6 +3011,7 @@
         <v>36</v>
       </c>
     </row>
+    <row r="44"/>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
@@ -2933,6 +3028,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
@@ -2941,15 +3037,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2970,10 +3069,20 @@
       </c>
       <c r="D1" s="6" t="inlineStr">
         <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Historical mean</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
           <t>Acceptance</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -2995,10 +3104,16 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>nM</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>5-50 nM</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3020,10 +3135,18 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>within 3-fold of historical mean</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
+          <t>µM</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>0.5-2 x historical mean</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3045,10 +3168,18 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>within 3-fold of historical mean</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
+          <t>µM</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>0.5-2 x historical mean</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3070,10 +3201,18 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>within 3-fold of historical mean</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
+          <t>µM</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>0.5-2 x historical mean</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3095,10 +3234,18 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>within 3-fold of historical mean</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
+          <t>µM</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>0.5-2 x historical mean</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3120,23 +3267,33 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>within 3-fold of historical mean</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
+          <t>µM</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>0.5-2 x historical mean</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>All runs met plate acceptance criteria. Checked by Ines Alvarado.</t>
+          <t>All accepted runs met plate acceptance criteria; rejected runs were repeated as noted on the hERG sheet. Checked by Ines Alvarado.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>